<commit_message>
Pengumpulan hasil Pilot dari dua coder dan rencana Pilot CC (lanjutan)
</commit_message>
<xml_diff>
--- a/P4 Pengembangan Kebutuhan Perangkat Lunak/A Elisitasi/A4 Coding/[3] Lembar_Coding_Codebook_1_0_3.xlsx
+++ b/P4 Pengembangan Kebutuhan Perangkat Lunak/A Elisitasi/A4 Coding/[3] Lembar_Coding_Codebook_1_0_3.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="361">
   <si>
     <t xml:space="preserve">Lembar Coding: Analisis Isi Krippendorff</t>
   </si>
@@ -53,7 +53,7 @@
     <t>2</t>
   </si>
   <si>
-    <t xml:space="preserve">Tentukan V4 Subjek Norma terlebih dahulu (Bagian 7.1), lalu V5 Relevansi dengan Uji Implikasi (Bagian 6 dan 7.2).</t>
+    <t xml:space="preserve">Tentukan V4 Subjek Norma terlebih dahulu dengan memeriksa berurutan S1 sampai S9 (Bagian 7.1), lalu V5 Relevansi dengan Uji Implikasi (Bagian 6 dan 7.2).</t>
   </si>
   <si>
     <t>3</t>
@@ -188,7 +188,7 @@
     <t>Kode</t>
   </si>
   <si>
-    <t xml:space="preserve">V4 S1 | V5 R2 | V6 T08 | V7 P2 | V8 F6 | V9 K3. Alasan: kewajiban dengan batas waktu yang dapat diuji.</t>
+    <t xml:space="preserve">V4 S2 | V5 R2 | V6 T08 | V7 P2 | V8 F6 | V9 K3. Alasan: kewajiban dengan batas waktu yang dapat diuji.</t>
   </si>
   <si>
     <t xml:space="preserve">Rujukan (Pasal atau Paragraf dan Kalimat)</t>
@@ -212,6 +212,9 @@
     <t>Bagian</t>
   </si>
   <si>
+    <t>CC</t>
+  </si>
+  <si>
     <t>Ya</t>
   </si>
   <si>
@@ -230,19 +233,19 @@
     <t>S1</t>
   </si>
   <si>
+    <t xml:space="preserve">Pengendali dan Prosesor</t>
+  </si>
+  <si>
+    <t>S2</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pengendali Data Pribadi</t>
   </si>
   <si>
-    <t>S2</t>
+    <t>S3</t>
   </si>
   <si>
     <t xml:space="preserve">Prosesor Data Pribadi</t>
-  </si>
-  <si>
-    <t>S3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pengendali dan Prosesor</t>
   </si>
   <si>
     <t>S4</t>
@@ -2154,7 +2157,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" ht="60" hidden="1" customHeight="1">
+    <row r="2" ht="60" customHeight="1">
       <c r="A2" s="16">
         <v>2</v>
       </c>
@@ -2183,7 +2186,9 @@
       <c r="L2" s="19"/>
       <c r="M2" s="20"/>
       <c r="N2" s="20"/>
-      <c r="O2" s="16"/>
+      <c r="O2" s="16" t="s">
+        <v>62</v>
+      </c>
       <c r="P2" s="18" t="str">
         <f t="shared" ref="P2:P9" si="0">IF(COUNTA(F2:K2)=6,"Lengkap","Belum lengkap ("&amp;(6-COUNTA(F2:K2))&amp;")")</f>
         <v xml:space="preserve">Belum lengkap (6)</v>
@@ -2671,7 +2676,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="13" ht="60" customHeight="1">
+    <row r="13" ht="60" hidden="1" customHeight="1">
       <c r="A13" s="16">
         <v>13</v>
       </c>
@@ -2701,7 +2706,7 @@
       <c r="M13" s="20"/>
       <c r="N13" s="20"/>
       <c r="O13" s="16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="P13" s="18" t="str">
         <f t="shared" si="2"/>
@@ -2767,7 +2772,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="15" ht="60" hidden="1" customHeight="1">
+    <row r="15" ht="60" customHeight="1">
       <c r="A15" s="16">
         <v>15</v>
       </c>
@@ -2796,7 +2801,9 @@
       <c r="L15" s="19"/>
       <c r="M15" s="20"/>
       <c r="N15" s="20"/>
-      <c r="O15" s="16"/>
+      <c r="O15" s="16" t="s">
+        <v>62</v>
+      </c>
       <c r="P15" s="18" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">Belum lengkap (6)</v>
@@ -3049,7 +3056,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="21" ht="60" customHeight="1">
+    <row r="21" ht="60" hidden="1" customHeight="1">
       <c r="A21" s="16">
         <v>21</v>
       </c>
@@ -3079,7 +3086,7 @@
       <c r="M21" s="20"/>
       <c r="N21" s="20"/>
       <c r="O21" s="16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="P21" s="18" t="str">
         <f t="shared" si="2"/>
@@ -3098,7 +3105,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="22" ht="60" hidden="1" customHeight="1">
+    <row r="22" ht="60" customHeight="1">
       <c r="A22" s="16">
         <v>22</v>
       </c>
@@ -3127,7 +3134,9 @@
       <c r="L22" s="19"/>
       <c r="M22" s="20"/>
       <c r="N22" s="20"/>
-      <c r="O22" s="16"/>
+      <c r="O22" s="16" t="s">
+        <v>62</v>
+      </c>
       <c r="P22" s="18" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">Belum lengkap (6)</v>
@@ -3239,7 +3248,7 @@
         <v xml:space="preserve">5. Pentingnya Perlindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="25" ht="60" customHeight="1">
+    <row r="25" ht="60" hidden="1" customHeight="1">
       <c r="A25" s="16">
         <v>25</v>
       </c>
@@ -3269,7 +3278,7 @@
       <c r="M25" s="20"/>
       <c r="N25" s="20"/>
       <c r="O25" s="16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="P25" s="18" t="str">
         <f t="shared" si="2"/>
@@ -3384,7 +3393,7 @@
 Identitas Anak</v>
       </c>
     </row>
-    <row r="28" ht="60" hidden="1" customHeight="1">
+    <row r="28" ht="60" customHeight="1">
       <c r="A28" s="16">
         <v>28</v>
       </c>
@@ -3413,7 +3422,9 @@
       <c r="L28" s="19"/>
       <c r="M28" s="20"/>
       <c r="N28" s="20"/>
-      <c r="O28" s="16"/>
+      <c r="O28" s="16" t="s">
+        <v>62</v>
+      </c>
       <c r="P28" s="18" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">Belum lengkap (6)</v>
@@ -3480,7 +3491,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="60" customHeight="1">
+    <row r="30" ht="60" hidden="1" customHeight="1">
       <c r="A30" s="16">
         <v>30</v>
       </c>
@@ -3510,7 +3521,7 @@
       <c r="M30" s="20"/>
       <c r="N30" s="20"/>
       <c r="O30" s="16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="P30" s="18" t="str">
         <f t="shared" si="2"/>
@@ -3578,7 +3589,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" ht="60" hidden="1" customHeight="1">
+    <row r="32" ht="60" customHeight="1">
       <c r="A32" s="16">
         <v>32</v>
       </c>
@@ -3607,7 +3618,9 @@
       <c r="L32" s="19"/>
       <c r="M32" s="20"/>
       <c r="N32" s="20"/>
-      <c r="O32" s="16"/>
+      <c r="O32" s="16" t="s">
+        <v>62</v>
+      </c>
       <c r="P32" s="18" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">Belum lengkap (6)</v>
@@ -3722,7 +3735,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" ht="60" customHeight="1">
+    <row r="35" ht="60" hidden="1" customHeight="1">
       <c r="A35" s="16">
         <v>35</v>
       </c>
@@ -3752,7 +3765,7 @@
       <c r="M35" s="20"/>
       <c r="N35" s="20"/>
       <c r="O35" s="16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="P35" s="18" t="str">
         <f t="shared" si="2"/>
@@ -4060,7 +4073,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="60" customHeight="1">
+    <row r="42" ht="60" hidden="1" customHeight="1">
       <c r="A42" s="16">
         <v>42</v>
       </c>
@@ -4090,7 +4103,7 @@
       <c r="M42" s="20"/>
       <c r="N42" s="20"/>
       <c r="O42" s="16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="P42" s="18" t="str">
         <f t="shared" si="2"/>
@@ -4158,7 +4171,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="60" customHeight="1">
+    <row r="44" ht="60" hidden="1" customHeight="1">
       <c r="A44" s="16">
         <v>44</v>
       </c>
@@ -4188,7 +4201,7 @@
       <c r="M44" s="20"/>
       <c r="N44" s="20"/>
       <c r="O44" s="16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="P44" s="18" t="str">
         <f t="shared" si="2"/>
@@ -4401,7 +4414,7 @@
         <v xml:space="preserve">Bagian Kedua Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="49" ht="60" hidden="1" customHeight="1">
+    <row r="49" ht="60" customHeight="1">
       <c r="A49" s="16">
         <v>49</v>
       </c>
@@ -4430,7 +4443,9 @@
       <c r="L49" s="19"/>
       <c r="M49" s="20"/>
       <c r="N49" s="20"/>
-      <c r="O49" s="16"/>
+      <c r="O49" s="16" t="s">
+        <v>62</v>
+      </c>
       <c r="P49" s="18" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">Belum lengkap (6)</v>
@@ -4545,7 +4560,7 @@
         <v xml:space="preserve">Bagian Kedua Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="52" ht="60" customHeight="1">
+    <row r="52" ht="60" hidden="1" customHeight="1">
       <c r="A52" s="16">
         <v>52</v>
       </c>
@@ -4575,7 +4590,7 @@
       <c r="M52" s="20"/>
       <c r="N52" s="20"/>
       <c r="O52" s="16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="P52" s="18" t="str">
         <f t="shared" si="2"/>
@@ -4643,7 +4658,7 @@
         <v xml:space="preserve">Bagian Kedua Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="54" ht="60" customHeight="1">
+    <row r="54" ht="60" hidden="1" customHeight="1">
       <c r="A54" s="16">
         <v>54</v>
       </c>
@@ -4673,7 +4688,7 @@
       <c r="M54" s="20"/>
       <c r="N54" s="20"/>
       <c r="O54" s="16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="P54" s="18" t="str">
         <f t="shared" si="2"/>
@@ -4693,7 +4708,7 @@
         <v xml:space="preserve">Bagian Kedua Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="55" ht="60" hidden="1" customHeight="1">
+    <row r="55" ht="60" customHeight="1">
       <c r="A55" s="16">
         <v>55</v>
       </c>
@@ -4722,7 +4737,9 @@
       <c r="L55" s="19"/>
       <c r="M55" s="20"/>
       <c r="N55" s="20"/>
-      <c r="O55" s="16"/>
+      <c r="O55" s="16" t="s">
+        <v>62</v>
+      </c>
       <c r="P55" s="18" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">Belum lengkap (6)</v>
@@ -4741,7 +4758,7 @@
         <v xml:space="preserve">Bagian Kedua Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="56" ht="60" customHeight="1">
+    <row r="56" ht="60" hidden="1" customHeight="1">
       <c r="A56" s="16">
         <v>56</v>
       </c>
@@ -4771,7 +4788,7 @@
       <c r="M56" s="20"/>
       <c r="N56" s="20"/>
       <c r="O56" s="16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="P56" s="18" t="str">
         <f t="shared" si="2"/>
@@ -5032,7 +5049,7 @@
 Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="62" ht="60" hidden="1" customHeight="1">
+    <row r="62" ht="60" customHeight="1">
       <c r="A62" s="16">
         <v>62</v>
       </c>
@@ -5061,7 +5078,9 @@
       <c r="L62" s="19"/>
       <c r="M62" s="20"/>
       <c r="N62" s="20"/>
-      <c r="O62" s="16"/>
+      <c r="O62" s="16" t="s">
+        <v>62</v>
+      </c>
       <c r="P62" s="18" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">Belum lengkap (6)</v>
@@ -5277,7 +5296,7 @@
 Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="67" ht="60" hidden="1" customHeight="1">
+    <row r="67" ht="60" customHeight="1">
       <c r="A67" s="16">
         <v>67</v>
       </c>
@@ -5306,7 +5325,9 @@
       <c r="L67" s="19"/>
       <c r="M67" s="20"/>
       <c r="N67" s="20"/>
-      <c r="O67" s="16"/>
+      <c r="O67" s="16" t="s">
+        <v>62</v>
+      </c>
       <c r="P67" s="18" t="str">
         <f t="shared" si="2"/>
         <v xml:space="preserve">Belum lengkap (6)</v>
@@ -5424,7 +5445,7 @@
 Kewajiban Pengendali Data Pribadi</v>
       </c>
     </row>
-    <row r="70" ht="60" customHeight="1">
+    <row r="70" ht="60" hidden="1" customHeight="1">
       <c r="A70" s="16">
         <v>70</v>
       </c>
@@ -5454,7 +5475,7 @@
       <c r="M70" s="20"/>
       <c r="N70" s="20"/>
       <c r="O70" s="16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="P70" s="18" t="str">
         <f t="shared" si="2"/>
@@ -5867,7 +5888,7 @@
 Kewajiban Prosesor Data Pribadi</v>
       </c>
     </row>
-    <row r="79" ht="60" customHeight="1">
+    <row r="79" ht="60" hidden="1" customHeight="1">
       <c r="A79" s="16">
         <v>79</v>
       </c>
@@ -5897,7 +5918,7 @@
       <c r="M79" s="20"/>
       <c r="N79" s="20"/>
       <c r="O79" s="16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="P79" s="18" t="str">
         <f t="shared" si="4"/>
@@ -5967,7 +5988,7 @@
 Pejabat atau Petugas yang Melaksanakan Fungsi Pelindungan Data Pribadi</v>
       </c>
     </row>
-    <row r="81" ht="60" customHeight="1">
+    <row r="81" ht="60" hidden="1" customHeight="1">
       <c r="A81" s="16">
         <v>81</v>
       </c>
@@ -5997,7 +6018,7 @@
       <c r="M81" s="20"/>
       <c r="N81" s="20"/>
       <c r="O81" s="16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="P81" s="18" t="str">
         <f t="shared" si="4"/>
@@ -6064,7 +6085,7 @@
         <v xml:space="preserve">Bagian Kedua</v>
       </c>
     </row>
-    <row r="83" ht="60" hidden="1" customHeight="1">
+    <row r="83" ht="60" customHeight="1">
       <c r="A83" s="16">
         <v>83</v>
       </c>
@@ -6093,7 +6114,9 @@
       <c r="L83" s="19"/>
       <c r="M83" s="20"/>
       <c r="N83" s="20"/>
-      <c r="O83" s="16"/>
+      <c r="O83" s="16" t="s">
+        <v>62</v>
+      </c>
       <c r="P83" s="18" t="str">
         <f t="shared" si="4"/>
         <v xml:space="preserve">Belum lengkap (6)</v>
@@ -6208,7 +6231,7 @@
         <v/>
       </c>
     </row>
-    <row r="86" ht="60" hidden="1" customHeight="1">
+    <row r="86" ht="60" customHeight="1">
       <c r="A86" s="16">
         <v>86</v>
       </c>
@@ -6237,7 +6260,9 @@
       <c r="L86" s="19"/>
       <c r="M86" s="20"/>
       <c r="N86" s="20"/>
-      <c r="O86" s="16"/>
+      <c r="O86" s="16" t="s">
+        <v>62</v>
+      </c>
       <c r="P86" s="18" t="str">
         <f t="shared" si="4"/>
         <v xml:space="preserve">Belum lengkap (6)</v>
@@ -6260,9 +6285,9 @@
   </sheetData>
   <autoFilter ref="A1:S86">
     <filterColumn colId="14">
-      <customFilters and="1">
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
+      <filters>
+        <filter val="CC"/>
+      </filters>
     </filterColumn>
   </autoFilter>
   <dataValidations count="2" disablePrompts="0">
@@ -6328,7 +6353,7 @@
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="8" disablePrompts="0">
-        <x14:dataValidation xr:uid="{0B7D02BB-579D-4249-AB9C-E797E755CA17}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kodekan pihak yang secara eksplisit menjadi subjek tata bahasa norma utama pada kolom “Isi”. Jangan menyimpulkan subjek dari judul BAB." showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{49FB9E35-2CFD-43A0-A247-DB745E892D46}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kodekan pihak yang secara eksplisit menjadi subjek tata bahasa norma utama pada kolom “Isi”.&#10;Pilih kode berurutan dan berhenti pada Subjek Norma pertama yang dianggap sesuai (S1 &gt; S2 &gt; S3 &gt; S4 &gt; S5 &gt; S6 &gt; S7 &gt; S8 &gt; S9)." promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$5:$D$13</xm:f>
           </x14:formula1>
@@ -6337,7 +6362,7 @@
           </x14:formula2>
           <xm:sqref>F3:F86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{53104D88-13E1-436B-AE40-E46BCD71630B}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tentukan dengan Uji Implikasi Bagian 6." showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{0C2737F5-A8E3-4764-B3EB-D3F8F3457204}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tentukan dengan Uji Implikasi Bagian 6." showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$16:$D$18</xm:f>
           </x14:formula1>
@@ -6346,7 +6371,7 @@
           </x14:formula2>
           <xm:sqref>G2:G86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{64F16F58-5BDC-439B-860D-A27831FAA83C}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Pilih satu tema dominan dari pohon keputusan Bagian 7.3. Pemilihan T99 wajib dijelaskan di V12." showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{13160206-E61E-46E1-B84B-410EE468C169}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Pilih satu tema dominan dari pohon keputusan Bagian 7.3. Pemilihan T99 wajib dijelaskan di V12." showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$21:$D$37</xm:f>
           </x14:formula1>
@@ -6355,7 +6380,7 @@
           </x14:formula2>
           <xm:sqref>H2:H86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{55094AFE-C663-46D9-8D47-FFC1DEE616A8}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Lihat Bagian 7.4" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{69049C8D-6EF6-4066-A02E-3D41A29CCAD0}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Lihat Bagian 7.4" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$40:$D$47</xm:f>
           </x14:formula1>
@@ -6364,7 +6389,7 @@
           </x14:formula2>
           <xm:sqref>I2:I86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{7B1586FE-619E-4789-9A69-DE6DD4ABDF37}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tahap siklus data yang terkait dari awal hingga akhir. Lihat Bagian 7.5" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{55AF09E2-D7BF-46B3-B147-AA863F9DCCB2}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tahap siklus data yang terkait dari awal hingga akhir. Lihat Bagian 7.5" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$50:$D$57</xm:f>
           </x14:formula1>
@@ -6373,7 +6398,7 @@
           </x14:formula2>
           <xm:sqref>J2:J86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{5DC7CEB6-6F37-4313-8251-44B6C976B072}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kandidat jenis kebutuhan SRS diperiksa berurutan K1 -&gt; K2 -&gt; K3 -&gt; K4 -&gt; K5. Lihat Bagian 7.6" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{0FC2F9A2-34D2-4AD0-9083-1D1191017953}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kandidat jenis kebutuhan SRS diperiksa berurutan K1 &gt; K2 &gt; K3 &gt; K4 &gt; K5. Lihat Bagian 7.6" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$60:$D$64</xm:f>
           </x14:formula1>
@@ -6382,7 +6407,7 @@
           </x14:formula2>
           <xm:sqref>K2:K86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{342CABB2-F4AE-47D5-B28B-F6D54CD4BB62}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tema kedua bila unit memuat dua tema (gunakan kode dari Bagian 7.3). T99 tidak digunakan di sini." promptTitle="Opsional" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{0845C06A-B707-4249-90D0-358711D723DB}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Tema kedua bila unit memuat dua tema (gunakan kode dari Bagian 7.3). T99 tidak digunakan di sini." promptTitle="Opsional" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$21:$D$36</xm:f>
           </x14:formula1>
@@ -6391,7 +6416,7 @@
           </x14:formula2>
           <xm:sqref>L2:L86</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{1924A37D-A0B9-4F01-AB06-22DF74F68B53}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kodekan pihak yang secara eksplisit menjadi subjek tata bahasa norma utama pada kolom “Isi”. Jangan menyimpulkan subjek dari judul BAB." promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{258FA0A7-5505-419A-975A-4C45E18CE2AD}" type="list" allowBlank="1" error="Pilih kode dari daftar (lihat sheet Daftar Kode)." errorStyle="stop" errorTitle="Kode tidak sah" imeMode="noControl" operator="between" prompt="Kodekan pihak yang secara eksplisit menjadi subjek tata bahasa norma utama pada kolom “Isi”. Jangan menyimpulkan subjek dari judul BAB." promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>'Daftar Kode'!$D$5:$D$13</xm:f>
           </x14:formula1>
@@ -6423,23 +6448,23 @@
   <sheetData>
     <row r="1" ht="16.5">
       <c r="A1" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" ht="15">
       <c r="A2" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" ht="15">
       <c r="A4" s="14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B4" s="14" t="s">
         <v>53</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D4" s="22" t="str">
         <f t="shared" ref="D4:D9" si="6">$B4 &amp; " - " &amp; $C4</f>
@@ -6451,14 +6476,14 @@
         <v>32</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D5" s="21" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve">S1 - Pengendali Data Pribadi</v>
+        <v xml:space="preserve">S1 - Pengendali dan Prosesor</v>
       </c>
     </row>
     <row r="6" ht="15">
@@ -6466,14 +6491,14 @@
         <v>32</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D6" s="21" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve">S2 - Prosesor Data Pribadi</v>
+        <v xml:space="preserve">S2 - Pengendali Data Pribadi</v>
       </c>
     </row>
     <row r="7" ht="15">
@@ -6481,14 +6506,14 @@
         <v>32</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D7" s="21" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve">S3 - Pengendali dan Prosesor</v>
+        <v xml:space="preserve">S3 - Prosesor Data Pribadi</v>
       </c>
     </row>
     <row r="8" ht="15">
@@ -6496,10 +6521,10 @@
         <v>32</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D8" s="21" t="str">
         <f t="shared" si="6"/>
@@ -6511,10 +6536,10 @@
         <v>32</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D9" s="21" t="str">
         <f t="shared" si="6"/>
@@ -6526,10 +6551,10 @@
         <v>32</v>
       </c>
       <c r="B10" s="24" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D10" s="21" t="str">
         <f t="shared" ref="D10:D64" si="7">$B10 &amp; " - " &amp; $C10</f>
@@ -6541,10 +6566,10 @@
         <v>32</v>
       </c>
       <c r="B11" s="24" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D11" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6556,10 +6581,10 @@
         <v>32</v>
       </c>
       <c r="B12" s="24" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D12" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6571,10 +6596,10 @@
         <v>32</v>
       </c>
       <c r="B13" s="24" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D13" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6583,13 +6608,13 @@
     </row>
     <row r="15" ht="15">
       <c r="A15" s="14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B15" s="14" t="s">
         <v>53</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D15" s="22" t="str">
         <f t="shared" si="7"/>
@@ -6601,10 +6626,10 @@
         <v>34</v>
       </c>
       <c r="B16" s="24" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D16" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6616,10 +6641,10 @@
         <v>34</v>
       </c>
       <c r="B17" s="24" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D17" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6631,10 +6656,10 @@
         <v>34</v>
       </c>
       <c r="B18" s="24" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D18" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6643,13 +6668,13 @@
     </row>
     <row r="20" ht="15">
       <c r="A20" s="14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B20" s="14" t="s">
         <v>53</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D20" s="22" t="str">
         <f t="shared" si="7"/>
@@ -6661,10 +6686,10 @@
         <v>36</v>
       </c>
       <c r="B21" s="24" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D21" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6676,10 +6701,10 @@
         <v>36</v>
       </c>
       <c r="B22" s="24" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D22" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6691,10 +6716,10 @@
         <v>36</v>
       </c>
       <c r="B23" s="24" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C23" s="23" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D23" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6706,10 +6731,10 @@
         <v>36</v>
       </c>
       <c r="B24" s="24" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D24" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6721,10 +6746,10 @@
         <v>36</v>
       </c>
       <c r="B25" s="24" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C25" s="23" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D25" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6736,10 +6761,10 @@
         <v>36</v>
       </c>
       <c r="B26" s="24" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D26" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6751,10 +6776,10 @@
         <v>36</v>
       </c>
       <c r="B27" s="24" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C27" s="23" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D27" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6766,10 +6791,10 @@
         <v>36</v>
       </c>
       <c r="B28" s="24" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D28" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6781,10 +6806,10 @@
         <v>36</v>
       </c>
       <c r="B29" s="24" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C29" s="23" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D29" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6796,10 +6821,10 @@
         <v>36</v>
       </c>
       <c r="B30" s="24" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C30" s="23" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D30" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6811,10 +6836,10 @@
         <v>36</v>
       </c>
       <c r="B31" s="24" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C31" s="23" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D31" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6826,10 +6851,10 @@
         <v>36</v>
       </c>
       <c r="B32" s="24" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C32" s="23" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D32" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6841,10 +6866,10 @@
         <v>36</v>
       </c>
       <c r="B33" s="24" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C33" s="23" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D33" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6856,10 +6881,10 @@
         <v>36</v>
       </c>
       <c r="B34" s="24" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C34" s="23" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D34" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6871,10 +6896,10 @@
         <v>36</v>
       </c>
       <c r="B35" s="24" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C35" s="23" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D35" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6886,10 +6911,10 @@
         <v>36</v>
       </c>
       <c r="B36" s="24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C36" s="23" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D36" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6901,10 +6926,10 @@
         <v>36</v>
       </c>
       <c r="B37" s="24" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C37" s="23" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D37" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6913,13 +6938,13 @@
     </row>
     <row r="39" ht="15">
       <c r="A39" s="14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B39" s="14" t="s">
         <v>53</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D39" s="22" t="str">
         <f t="shared" si="7"/>
@@ -6931,10 +6956,10 @@
         <v>38</v>
       </c>
       <c r="B40" s="24" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C40" s="23" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D40" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6946,10 +6971,10 @@
         <v>38</v>
       </c>
       <c r="B41" s="24" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D41" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6961,10 +6986,10 @@
         <v>38</v>
       </c>
       <c r="B42" s="24" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C42" s="23" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D42" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6976,10 +7001,10 @@
         <v>38</v>
       </c>
       <c r="B43" s="24" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D43" s="21" t="str">
         <f t="shared" si="7"/>
@@ -6991,10 +7016,10 @@
         <v>38</v>
       </c>
       <c r="B44" s="24" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C44" s="23" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D44" s="21" t="str">
         <f t="shared" si="7"/>
@@ -7006,10 +7031,10 @@
         <v>38</v>
       </c>
       <c r="B45" s="24" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C45" s="23" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D45" s="21" t="str">
         <f t="shared" si="7"/>
@@ -7021,10 +7046,10 @@
         <v>38</v>
       </c>
       <c r="B46" s="24" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C46" s="23" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D46" s="21" t="str">
         <f t="shared" si="7"/>
@@ -7036,10 +7061,10 @@
         <v>38</v>
       </c>
       <c r="B47" s="24" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C47" s="23" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D47" s="21" t="str">
         <f t="shared" si="7"/>
@@ -7048,13 +7073,13 @@
     </row>
     <row r="49" ht="15">
       <c r="A49" s="14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B49" s="14" t="s">
         <v>53</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D49" s="22" t="str">
         <f t="shared" si="7"/>
@@ -7066,10 +7091,10 @@
         <v>40</v>
       </c>
       <c r="B50" s="24" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C50" s="23" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D50" s="21" t="str">
         <f t="shared" si="7"/>
@@ -7081,10 +7106,10 @@
         <v>40</v>
       </c>
       <c r="B51" s="24" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C51" s="23" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D51" s="21" t="str">
         <f t="shared" si="7"/>
@@ -7096,10 +7121,10 @@
         <v>40</v>
       </c>
       <c r="B52" s="24" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C52" s="23" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D52" s="21" t="str">
         <f t="shared" si="7"/>
@@ -7111,10 +7136,10 @@
         <v>40</v>
       </c>
       <c r="B53" s="24" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C53" s="23" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D53" s="21" t="str">
         <f t="shared" si="7"/>
@@ -7126,10 +7151,10 @@
         <v>40</v>
       </c>
       <c r="B54" s="24" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C54" s="23" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D54" s="21" t="str">
         <f t="shared" si="7"/>
@@ -7141,10 +7166,10 @@
         <v>40</v>
       </c>
       <c r="B55" s="24" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C55" s="23" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D55" s="21" t="str">
         <f t="shared" si="7"/>
@@ -7156,10 +7181,10 @@
         <v>40</v>
       </c>
       <c r="B56" s="24" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C56" s="23" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D56" s="21" t="str">
         <f t="shared" si="7"/>
@@ -7171,10 +7196,10 @@
         <v>40</v>
       </c>
       <c r="B57" s="24" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C57" s="23" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D57" s="21" t="str">
         <f t="shared" si="7"/>
@@ -7183,13 +7208,13 @@
     </row>
     <row r="59" ht="15">
       <c r="A59" s="14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B59" s="14" t="s">
         <v>53</v>
       </c>
       <c r="C59" s="14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D59" s="22" t="str">
         <f t="shared" si="7"/>
@@ -7201,10 +7226,10 @@
         <v>42</v>
       </c>
       <c r="B60" s="24" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C60" s="23" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D60" s="21" t="str">
         <f t="shared" si="7"/>
@@ -7216,10 +7241,10 @@
         <v>42</v>
       </c>
       <c r="B61" s="24" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C61" s="23" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D61" s="21" t="str">
         <f t="shared" si="7"/>
@@ -7231,10 +7256,10 @@
         <v>42</v>
       </c>
       <c r="B62" s="24" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C62" s="23" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D62" s="21" t="str">
         <f t="shared" si="7"/>
@@ -7246,10 +7271,10 @@
         <v>42</v>
       </c>
       <c r="B63" s="24" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C63" s="23" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D63" s="21" t="str">
         <f t="shared" si="7"/>
@@ -7261,10 +7286,10 @@
         <v>42</v>
       </c>
       <c r="B64" s="24" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C64" s="23" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D64" s="21" t="str">
         <f t="shared" si="7"/>
@@ -7294,7 +7319,7 @@
   <sheetData>
     <row r="1" ht="15">
       <c r="A1" s="25" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B1" s="25" t="s">
         <v>60</v>
@@ -7303,1484 +7328,1484 @@
         <v>61</v>
       </c>
       <c r="D1" s="25" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E1" s="25" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F1" s="25" t="s">
         <v>56</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2" ht="15">
       <c r="A2" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" ht="15">
       <c r="A3" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="4" ht="15">
       <c r="A4" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="5" ht="15">
       <c r="A5" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="6" ht="15">
       <c r="A6" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="7" ht="15">
       <c r="A7" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="8" ht="15">
       <c r="A8" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="9" ht="15">
       <c r="A9" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="10" ht="15">
       <c r="A10" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="11" ht="15">
       <c r="A11" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="12" ht="15">
       <c r="A12" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="13" ht="15">
       <c r="A13" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="14" ht="15">
       <c r="A14" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="15" ht="15">
       <c r="A15" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="16" ht="15">
       <c r="A16" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="17" ht="15">
       <c r="A17" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="18" ht="15">
       <c r="A18" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="19" ht="15">
       <c r="A19" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="20" ht="15">
       <c r="A20" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="21" ht="15">
       <c r="A21" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="22" ht="15">
       <c r="A22" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="23" ht="15">
       <c r="A23" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="24" ht="15">
       <c r="A24" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="25" ht="15">
       <c r="A25" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="26" ht="15">
       <c r="A26" s="11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="27" ht="55.200000000000003">
       <c r="A27" s="11" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="28" ht="55.200000000000003">
       <c r="A28" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="29" ht="55.200000000000003">
       <c r="A29" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="30" ht="28.350000000000001">
       <c r="A30" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="31" ht="55.200000000000003">
       <c r="A31" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="32" ht="68.650000000000006">
       <c r="A32" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="33" ht="68.650000000000006">
       <c r="A33" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="34" ht="68.650000000000006">
       <c r="A34" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="35" ht="68.650000000000006">
       <c r="A35" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="36" ht="68.650000000000006">
       <c r="A36" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="37" ht="68.650000000000006">
       <c r="A37" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="38" ht="68.650000000000006">
       <c r="A38" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="39" ht="68.650000000000006">
       <c r="A39" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B39" s="12" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="40" ht="68.650000000000006">
       <c r="A40" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B40" s="12" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="41" ht="68.650000000000006">
       <c r="A41" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B41" s="12" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="42" ht="68.650000000000006">
       <c r="A42" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B42" s="12" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="43" ht="68.650000000000006">
       <c r="A43" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="44" ht="68.650000000000006">
       <c r="A44" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B44" s="12" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="45" ht="68.650000000000006">
       <c r="A45" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B45" s="12" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="46" ht="216.40000000000001">
       <c r="A46" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B46" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E46" s="11" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="F46" s="11" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="47" ht="216.40000000000001">
       <c r="A47" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B47" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C47" s="11" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F47" s="11" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="48" ht="216.40000000000001">
       <c r="A48" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B48" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C48" s="11" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E48" s="11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="49" ht="216.40000000000001">
       <c r="A49" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B49" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C49" s="11" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="50" ht="216.40000000000001">
       <c r="A50" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B50" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C50" s="11" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E50" s="11" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="F50" s="11" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="51" ht="216.40000000000001">
       <c r="A51" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B51" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C51" s="11" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="52" ht="216.40000000000001">
       <c r="A52" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B52" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C52" s="11" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E52" s="11" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="53" ht="216.40000000000001">
       <c r="A53" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B53" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C53" s="11" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="54" ht="216.40000000000001">
       <c r="A54" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B54" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C54" s="11" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E54" s="11" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="55" ht="216.40000000000001">
       <c r="A55" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B55" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C55" s="11" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="56" ht="216.40000000000001">
       <c r="A56" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B56" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C56" s="11" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="57" ht="216.40000000000001">
       <c r="A57" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B57" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C57" s="11" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="58" ht="216.40000000000001">
       <c r="A58" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B58" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C58" s="11" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E58" s="11" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="59" ht="216.40000000000001">
       <c r="A59" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B59" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C59" s="11" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E59" s="11" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="60" ht="216.40000000000001">
       <c r="A60" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B60" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C60" s="11" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E60" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="61" ht="216.40000000000001">
       <c r="A61" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B61" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C61" s="12" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E61" s="11" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="62" ht="216.40000000000001">
       <c r="A62" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B62" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C62" s="12" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="63" ht="216.40000000000001">
       <c r="A63" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B63" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C63" s="12" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E63" s="11" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="64" ht="216.40000000000001">
       <c r="A64" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B64" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C64" s="12" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E64" s="11" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="F64" s="11" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="65" ht="216.40000000000001">
       <c r="A65" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B65" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C65" s="12" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E65" s="11" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="F65" s="11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="66" ht="216.40000000000001">
       <c r="A66" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B66" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C66" s="12" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E66" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F66" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="67" ht="216.40000000000001">
       <c r="A67" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B67" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C67" s="12" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E67" s="11" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="68" ht="216.40000000000001">
       <c r="A68" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B68" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C68" s="12" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E68" s="11" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="F68" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="69" ht="216.40000000000001">
       <c r="A69" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B69" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C69" s="12" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E69" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="70" ht="216.40000000000001">
       <c r="A70" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B70" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C70" s="12" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E70" s="11" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="F70" s="11" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="71" ht="216.40000000000001">
       <c r="A71" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B71" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C71" s="12" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E71" s="11" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="F71" s="11" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="72" ht="216.40000000000001">
       <c r="A72" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B72" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C72" s="12" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E72" s="11" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="F72" s="11" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="73" ht="216.40000000000001">
       <c r="A73" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B73" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C73" s="12" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E73" s="11" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F73" s="11" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="74" ht="216.40000000000001">
       <c r="A74" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B74" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C74" s="12" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E74" s="11" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="F74" s="11" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="75" ht="216.40000000000001">
       <c r="A75" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B75" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C75" s="12" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E75" s="11" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F75" s="11" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="76" ht="216.40000000000001">
       <c r="A76" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B76" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C76" s="12" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E76" s="11" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="F76" s="11" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="77" ht="216.40000000000001">
       <c r="A77" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B77" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C77" s="12" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E77" s="11" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F77" s="11" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="78" ht="216.40000000000001">
       <c r="A78" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B78" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C78" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E78" s="11" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F78" s="26" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="79" ht="216.40000000000001">
       <c r="A79" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B79" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C79" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E79" s="11" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="F79" s="11" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="80" ht="216.40000000000001">
       <c r="A80" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B80" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C80" s="12" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E80" s="11" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="F80" s="11" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="81" ht="162.65000000000001">
       <c r="A81" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B81" s="11" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C81" s="12" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="E81" s="11" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="F81" s="11" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="82" ht="15">
       <c r="A82" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B82" s="11" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C82" s="11" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="E82" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F82" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="83" ht="108.95">
       <c r="A83" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B83" s="12" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E83" s="11" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="F83" s="11" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="84" ht="108.95">
       <c r="A84" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B84" s="12" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E84" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="F84" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row r="85" ht="55.200000000000003">
       <c r="A85" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B85" s="12" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E85" s="11" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F85" s="11" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="86" ht="95.5">
       <c r="A86" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B86" s="12" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C86" s="12" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E86" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F86" s="11" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="87" ht="15">
       <c r="A87" s="11" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B87" s="11" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
   </sheetData>

</xml_diff>